<commit_message>
Finance : modèle Prévisions Pop Tables modifié par le responsable Finance (budget sur 36 mois, plan financier, prix et marges) (29/10/2026)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2 FINANCE/PREVISIONS/2026 1028 Modèle Pop Tables - Budget sur 36 mois, plan financier, prix et marges.xlsx
+++ b/2 FINANCE/PREVISIONS/2026 1028 Modèle Pop Tables - Budget sur 36 mois, plan financier, prix et marges.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vians\Documents\Claude\Projects\HEC-GEMM-Groupe-7\2 FINANCE\PREVISIONS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47501460-8397-4BCC-93DF-52AAF23A4E44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9484D665-FFFB-470F-8705-E8648B22E82C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" firstSheet="3" activeTab="3" xr2:uid="{09426CC5-4BCC-48B7-8854-C5C8E2CE30D1}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="1" xr2:uid="{09426CC5-4BCC-48B7-8854-C5C8E2CE30D1}"/>
   </bookViews>
   <sheets>
     <sheet name="Mode d'emploi" sheetId="1" r:id="rId1"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="473">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="475">
   <si>
     <t>Rubrique</t>
   </si>
@@ -1159,15 +1159,9 @@
     <t>Ville 2 (France)</t>
   </si>
   <si>
-    <t>Ville 3 (étranger)</t>
-  </si>
-  <si>
     <t>Étranger</t>
   </si>
   <si>
-    <t>Ville 4 (France)</t>
-  </si>
-  <si>
     <t>Ville 5 (étranger)</t>
   </si>
   <si>
@@ -1487,6 +1481,18 @@
   </si>
   <si>
     <t>Revu le 28/10/2026 (soir) par le responsable Finance : nouvelles villes actives dès novembre ; 40 privatisations par ville et par an dès l'année 2 ; coordinateurs (1 par événement hebdomadaire) et commerciaux (1 par ville active, dès l'année 3) calculés à partir de l'activité ; un manager en année 3 ; locaux et logiciels par poste payé ; prix et coûts revus dans « Prix et marges ». Décisions D-05, D-06, D-08, D-14, D-15, D-19 intégrées ; campagne de lancement (10 000 €), protection juridique et assurance (2 % du CA) et budget des ventes. Toutes les autres valeurs restent des hypothèses (H) : voir la fiche des données manquantes du 28/10/2026.</t>
+  </si>
+  <si>
+    <t>france</t>
+  </si>
+  <si>
+    <t>etranger</t>
+  </si>
+  <si>
+    <t>Ville 3 (france)</t>
+  </si>
+  <si>
+    <t>Ville 4 (Etranger)</t>
   </si>
 </sst>
 </file>
@@ -2234,12 +2240,12 @@
   <sheetData>
     <row r="1" spans="1:2" ht="18" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="13" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="13" x14ac:dyDescent="0.25">
@@ -2263,7 +2269,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="50" x14ac:dyDescent="0.25">
@@ -2271,7 +2277,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="25" x14ac:dyDescent="0.25">
@@ -2335,7 +2341,7 @@
         <v>20</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="25" x14ac:dyDescent="0.25">
@@ -2478,10 +2484,10 @@
         <v>117</v>
       </c>
       <c r="H7" s="21" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="I7" s="20" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="37.5" x14ac:dyDescent="0.25">
@@ -2507,7 +2513,7 @@
         <v>82</v>
       </c>
       <c r="H8" s="21" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="I8" s="20" t="s">
         <v>83</v>
@@ -3003,10 +3009,10 @@
         <v>117</v>
       </c>
       <c r="H26" s="21" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="I26" s="20" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -3183,7 +3189,7 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="18" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="B33" s="18" t="s">
         <v>51</v>
@@ -3204,10 +3210,10 @@
         <v>117</v>
       </c>
       <c r="H33" s="21" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="I33" s="20" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
     </row>
     <row r="34" spans="1:9" ht="13" x14ac:dyDescent="0.25">
@@ -4854,7 +4860,7 @@
         <v>275</v>
       </c>
       <c r="AP7" s="1" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
     </row>
     <row r="8" spans="1:43" ht="13" x14ac:dyDescent="0.3">
@@ -4985,7 +4991,7 @@
         <v>82</v>
       </c>
       <c r="AP8" s="1" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
     </row>
     <row r="9" spans="1:43" ht="13" x14ac:dyDescent="0.3">
@@ -5563,7 +5569,7 @@
         <v>82</v>
       </c>
       <c r="AP12" s="1" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
     </row>
     <row r="13" spans="1:43" ht="13" x14ac:dyDescent="0.3">
@@ -5729,7 +5735,7 @@
     </row>
     <row r="14" spans="1:43" ht="13" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="B14" s="13">
         <f t="shared" si="1"/>
@@ -5855,12 +5861,12 @@
         <v>82</v>
       </c>
       <c r="AP14" s="1" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
     </row>
     <row r="15" spans="1:43" ht="13" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="B15" s="13">
         <f t="shared" si="1"/>
@@ -5991,7 +5997,7 @@
     </row>
     <row r="16" spans="1:43" ht="13" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="B16" s="13">
         <f>SUM(E16:P16)</f>
@@ -6141,12 +6147,12 @@
         <v>117</v>
       </c>
       <c r="AP16" s="1" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
     </row>
     <row r="17" spans="1:43" ht="13" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="B17" s="13">
         <f>SUM(E17:P17)</f>
@@ -6296,7 +6302,7 @@
         <v>117</v>
       </c>
       <c r="AP17" s="1" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
     </row>
     <row r="18" spans="1:43" ht="13" x14ac:dyDescent="0.3">
@@ -6563,7 +6569,7 @@
     </row>
     <row r="20" spans="1:43" ht="13" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="B20" s="13">
         <f>MAX(E20:P20)</f>
@@ -6725,12 +6731,12 @@
         <v>117</v>
       </c>
       <c r="AP20" s="1" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
     </row>
     <row r="21" spans="1:43" ht="13" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="B21" s="13">
         <f>MAX(E21:P21)</f>
@@ -6892,12 +6898,12 @@
         <v>117</v>
       </c>
       <c r="AP21" s="1" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
     </row>
     <row r="22" spans="1:43" ht="13" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B22" s="13">
         <f>MAX(E22:P22)</f>
@@ -7059,7 +7065,7 @@
         <v>117</v>
       </c>
       <c r="AP22" s="1" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
     </row>
     <row r="23" spans="1:43" ht="13" x14ac:dyDescent="0.3">
@@ -8801,7 +8807,7 @@
         <v>117</v>
       </c>
       <c r="AP34" s="1" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="AQ34" s="55"/>
     </row>
@@ -8970,7 +8976,7 @@
         <v>117</v>
       </c>
       <c r="AP35" s="1" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="AQ35" s="55"/>
     </row>
@@ -9516,7 +9522,7 @@
         <v>117</v>
       </c>
       <c r="AP39" s="1" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="AQ39" s="57">
         <f>TVA!$C$30</f>
@@ -9687,7 +9693,7 @@
         <v>117</v>
       </c>
       <c r="AP40" s="1" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="AQ40" s="57">
         <f>TVA!$C$31</f>
@@ -11409,7 +11415,7 @@
         <v>117</v>
       </c>
       <c r="AP52" s="1" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="AQ52" s="57">
         <v>0.1</v>
@@ -14857,8 +14863,7 @@
         <v>336</v>
       </c>
       <c r="B78" s="16">
-        <f>SUM(E78:P78)</f>
-        <v>7000</v>
+        <v>70000</v>
       </c>
       <c r="C78" s="16">
         <f>SUM(Q78:AB78)</f>
@@ -14869,7 +14874,7 @@
         <v>0</v>
       </c>
       <c r="E78" s="14">
-        <v>7000</v>
+        <v>70000</v>
       </c>
       <c r="F78" s="14">
         <v>0</v>
@@ -14989,7 +14994,7 @@
       </c>
       <c r="B79" s="16">
         <f>SUM(E79:P79)</f>
-        <v>-8551.1785714285943</v>
+        <v>54448.821428571413</v>
       </c>
       <c r="C79" s="16">
         <f>SUM(Q79:AB79)</f>
@@ -15001,7 +15006,7 @@
       </c>
       <c r="E79" s="15">
         <f t="shared" ref="E79:AN79" si="36">E59-E64+E75+E77+E78</f>
-        <v>-17763</v>
+        <v>45237</v>
       </c>
       <c r="F79" s="15">
         <f t="shared" si="36"/>
@@ -15153,159 +15158,159 @@
       </c>
       <c r="B80" s="16">
         <f>P80</f>
-        <v>-8551.1785714285943</v>
+        <v>54448.821428571413</v>
       </c>
       <c r="C80" s="16">
         <f>AB80</f>
-        <v>433353.49647619051</v>
+        <v>496353.49647619051</v>
       </c>
       <c r="D80" s="16">
         <f>AN80</f>
-        <v>808460.35847619059</v>
+        <v>871460.35847619059</v>
       </c>
       <c r="E80" s="16">
         <f>E79</f>
-        <v>-17763</v>
+        <v>45237</v>
       </c>
       <c r="F80" s="16">
         <f t="shared" ref="F80:AN80" si="37">E80+F79</f>
-        <v>-11514.000000000002</v>
+        <v>51486</v>
       </c>
       <c r="G80" s="16">
         <f t="shared" si="37"/>
-        <v>-3016.6428571428605</v>
+        <v>59983.357142857145</v>
       </c>
       <c r="H80" s="16">
         <f t="shared" si="37"/>
-        <v>-13995.642857142862</v>
+        <v>49004.357142857145</v>
       </c>
       <c r="I80" s="16">
         <f t="shared" si="37"/>
-        <v>-52928.892857142862</v>
+        <v>10071.107142857145</v>
       </c>
       <c r="J80" s="16">
         <f t="shared" si="37"/>
-        <v>-38639.17857142858</v>
+        <v>24360.821428571428</v>
       </c>
       <c r="K80" s="16">
         <f t="shared" si="37"/>
-        <v>-36919.821428571442</v>
+        <v>26080.178571428565</v>
       </c>
       <c r="L80" s="16">
         <f t="shared" si="37"/>
-        <v>-34340.714285714304</v>
+        <v>28659.285714285703</v>
       </c>
       <c r="M80" s="16">
         <f t="shared" si="37"/>
-        <v>-44263.357142857159</v>
+        <v>18736.642857142848</v>
       </c>
       <c r="N80" s="16">
         <f t="shared" si="37"/>
-        <v>-35674.357142857159</v>
+        <v>27325.642857142848</v>
       </c>
       <c r="O80" s="16">
         <f t="shared" si="37"/>
-        <v>-40242.642857142877</v>
+        <v>22757.35714285713</v>
       </c>
       <c r="P80" s="16">
         <f t="shared" si="37"/>
-        <v>-8551.1785714285943</v>
+        <v>54448.821428571413</v>
       </c>
       <c r="Q80" s="16">
         <f t="shared" si="37"/>
-        <v>27445.629666666646</v>
+        <v>90445.629666666646</v>
       </c>
       <c r="R80" s="16">
         <f t="shared" si="37"/>
-        <v>69142.437904761886</v>
+        <v>132142.43790476187</v>
       </c>
       <c r="S80" s="16">
         <f t="shared" si="37"/>
-        <v>109803.04376190473</v>
+        <v>172803.04376190473</v>
       </c>
       <c r="T80" s="16">
         <f t="shared" si="37"/>
-        <v>146472.34009523806</v>
+        <v>209472.34009523806</v>
       </c>
       <c r="U80" s="16">
         <f t="shared" si="37"/>
-        <v>183141.63642857139</v>
+        <v>246141.63642857139</v>
       </c>
       <c r="V80" s="16">
         <f t="shared" si="37"/>
-        <v>219810.93276190473</v>
+        <v>282810.93276190473</v>
       </c>
       <c r="W80" s="16">
         <f t="shared" si="37"/>
-        <v>256480.22909523806</v>
+        <v>319480.22909523803</v>
       </c>
       <c r="X80" s="16">
         <f t="shared" si="37"/>
-        <v>293149.52542857139</v>
+        <v>356149.52542857139</v>
       </c>
       <c r="Y80" s="16">
         <f t="shared" si="37"/>
-        <v>282818.82176190475</v>
+        <v>345818.82176190475</v>
       </c>
       <c r="Z80" s="16">
         <f t="shared" si="37"/>
-        <v>342104.01095238095</v>
+        <v>405104.01095238095</v>
       </c>
       <c r="AA80" s="16">
         <f t="shared" si="37"/>
-        <v>364684.20014285715</v>
+        <v>427684.20014285715</v>
       </c>
       <c r="AB80" s="16">
         <f t="shared" si="37"/>
-        <v>433353.49647619051</v>
+        <v>496353.49647619051</v>
       </c>
       <c r="AC80" s="16">
         <f t="shared" si="37"/>
-        <v>460328.93438095244</v>
+        <v>523328.93438095244</v>
       </c>
       <c r="AD80" s="16">
         <f t="shared" si="37"/>
-        <v>494454.19371428579</v>
+        <v>557454.19371428574</v>
       </c>
       <c r="AE80" s="16">
         <f t="shared" si="37"/>
-        <v>527179.45304761908</v>
+        <v>590179.45304761908</v>
       </c>
       <c r="AF80" s="16">
         <f t="shared" si="37"/>
-        <v>559904.71238095243</v>
+        <v>622904.71238095243</v>
       </c>
       <c r="AG80" s="16">
         <f t="shared" si="37"/>
-        <v>592629.97171428578</v>
+        <v>655629.97171428578</v>
       </c>
       <c r="AH80" s="16">
         <f t="shared" si="37"/>
-        <v>625355.23104761913</v>
+        <v>688355.23104761913</v>
       </c>
       <c r="AI80" s="16">
         <f t="shared" si="37"/>
-        <v>658080.49038095248</v>
+        <v>721080.49038095248</v>
       </c>
       <c r="AJ80" s="16">
         <f t="shared" si="37"/>
-        <v>690805.74971428583</v>
+        <v>753805.74971428583</v>
       </c>
       <c r="AK80" s="16">
         <f t="shared" si="37"/>
-        <v>629531.00904761918</v>
+        <v>692531.00904761918</v>
       </c>
       <c r="AL80" s="16">
         <f t="shared" si="37"/>
-        <v>741258.05409523821</v>
+        <v>804258.05409523821</v>
       </c>
       <c r="AM80" s="16">
         <f t="shared" si="37"/>
-        <v>775735.09914285725</v>
+        <v>838735.09914285725</v>
       </c>
       <c r="AN80" s="16">
         <f t="shared" si="37"/>
-        <v>808460.35847619059</v>
+        <v>871460.35847619059</v>
       </c>
     </row>
     <row r="82" spans="1:43" ht="13" x14ac:dyDescent="0.3">
@@ -15436,46 +15441,46 @@
     </row>
     <row r="90" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="B90" s="71">
         <v>40</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
     </row>
     <row r="91" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="B91" s="71">
         <v>300</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
     </row>
     <row r="92" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B92" s="71">
         <v>80</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
     </row>
     <row r="93" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="B93" s="71">
         <v>50</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
     </row>
     <row r="95" spans="1:43" ht="26" x14ac:dyDescent="0.25">
@@ -15520,72 +15525,72 @@
         <v>46692</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
-        <v>363</v>
+        <v>473</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>364</v>
+        <v>471</v>
       </c>
       <c r="C98" s="52">
         <f>EDATE($B$3,12)</f>
         <v>46692</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
-        <v>365</v>
+        <v>474</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>360</v>
+        <v>472</v>
       </c>
       <c r="C99" s="52">
         <f>EDATE($B$3,24)</f>
         <v>47058</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C100" s="52">
         <f>EDATE($B$3,24)</f>
         <v>47058</v>
       </c>
       <c r="E100" s="1" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C101" s="52">
         <f>EDATE($B$3,24)</f>
         <v>47058</v>
       </c>
       <c r="E101" s="1" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
     </row>
     <row r="103" spans="1:5" ht="13" x14ac:dyDescent="0.3">
       <c r="A103" s="4" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
     </row>
   </sheetData>
@@ -15607,7 +15612,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="13" x14ac:dyDescent="0.3">
@@ -15861,7 +15866,7 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="B20" s="1">
         <v>33</v>
@@ -16021,7 +16026,7 @@
         <v>249</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="C30" s="41">
         <v>0.2</v>
@@ -16038,7 +16043,7 @@
         <v>250</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="C31" s="41">
         <v>0.2</v>
@@ -16055,7 +16060,7 @@
         <v>110</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="C32" s="41">
         <v>0.2</v>
@@ -16069,10 +16074,10 @@
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C33" s="41">
         <v>0</v>
@@ -16089,7 +16094,7 @@
         <v>253</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="C34" s="41">
         <v>0.2</v>
@@ -16106,7 +16111,7 @@
         <v>112</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="C35" s="41">
         <v>0</v>
@@ -16123,7 +16128,7 @@
         <v>113</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="C36" s="41">
         <v>0.1</v>
@@ -16140,7 +16145,7 @@
         <v>114</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C37" s="41">
         <v>0</v>
@@ -16154,10 +16159,10 @@
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="C38" s="41">
         <v>0.2</v>
@@ -16171,7 +16176,7 @@
     </row>
     <row r="40" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A40" s="60" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B40"/>
       <c r="C40"/>
@@ -16525,12 +16530,12 @@
   <sheetData>
     <row r="1" spans="1:14" ht="18" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="13" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="13" x14ac:dyDescent="0.3">
@@ -17254,7 +17259,7 @@
   <sheetData>
     <row r="1" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="59" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="B1"/>
       <c r="C1"/>
@@ -17268,7 +17273,7 @@
     </row>
     <row r="2" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A2" s="60" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="B2"/>
       <c r="C2"/>
@@ -17344,10 +17349,10 @@
     </row>
     <row r="7" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="B7" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="C7" s="66">
         <f>'Budget 36 mois'!B7</f>
@@ -17362,7 +17367,7 @@
         <v>6</v>
       </c>
       <c r="F7" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="G7"/>
       <c r="H7"/>
@@ -17371,10 +17376,10 @@
     </row>
     <row r="8" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="B8" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="C8" s="66">
         <f>'Budget 36 mois'!B11</f>
@@ -17389,7 +17394,7 @@
         <v>66</v>
       </c>
       <c r="F8" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
@@ -17398,10 +17403,10 @@
     </row>
     <row r="9" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="B9" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="C9" s="66">
         <f>'Budget 36 mois'!B8</f>
@@ -17423,10 +17428,10 @@
     </row>
     <row r="10" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B10" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="C10" s="66">
         <f>'Budget 36 mois'!B9</f>
@@ -17448,10 +17453,10 @@
     </row>
     <row r="11" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="B11" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="C11" s="66">
         <f>'Budget 36 mois'!B10</f>
@@ -17473,10 +17478,10 @@
     </row>
     <row r="12" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="B12" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="C12" s="66">
         <f>'Budget 36 mois'!B12</f>
@@ -17491,7 +17496,7 @@
         <v>240</v>
       </c>
       <c r="F12" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="G12"/>
       <c r="H12"/>
@@ -17503,7 +17508,7 @@
         <v>107</v>
       </c>
       <c r="B13" s="38" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="C13" s="69">
         <f>'Budget 36 mois'!B13</f>
@@ -17564,7 +17569,7 @@
     </row>
     <row r="16" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="B16" t="s">
         <v>51</v>
@@ -17629,7 +17634,7 @@
     </row>
     <row r="19" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="B19" t="s">
         <v>51</v>
@@ -17647,7 +17652,7 @@
         <v>643836.88800000015</v>
       </c>
       <c r="F19" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="G19"/>
       <c r="H19"/>
@@ -17681,7 +17686,7 @@
     </row>
     <row r="21" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="B21" t="s">
         <v>51</v>
@@ -17699,7 +17704,7 @@
         <v>0</v>
       </c>
       <c r="F21" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="G21"/>
       <c r="H21"/>
@@ -17708,7 +17713,7 @@
     </row>
     <row r="22" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="B22" t="s">
         <v>51</v>
@@ -17726,7 +17731,7 @@
         <v>29210.000000000004</v>
       </c>
       <c r="F22" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="G22"/>
       <c r="H22"/>
@@ -17735,7 +17740,7 @@
     </row>
     <row r="23" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B23" t="s">
         <v>51</v>
@@ -17785,7 +17790,7 @@
     </row>
     <row r="25" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="B25" t="s">
         <v>51</v>
@@ -17803,7 +17808,7 @@
         <v>76559.999999999971</v>
       </c>
       <c r="F25" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="G25"/>
       <c r="H25"/>
@@ -17862,7 +17867,7 @@
     </row>
     <row r="28" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A28" s="37" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B28" s="37"/>
       <c r="C28" s="37"/>
@@ -17876,7 +17881,7 @@
     </row>
     <row r="29" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B29" t="s">
         <v>51</v>
@@ -17901,7 +17906,7 @@
     </row>
     <row r="30" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="B30" t="s">
         <v>132</v>
@@ -17969,7 +17974,7 @@
         <v>212.59935743716258</v>
       </c>
       <c r="F32" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="G32"/>
       <c r="H32"/>
@@ -17990,7 +17995,7 @@
     </row>
     <row r="34" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A34" s="37" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="B34" s="37"/>
       <c r="C34" s="37"/>
@@ -18004,7 +18009,7 @@
     </row>
     <row r="35" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A35" s="38" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="B35" s="38" t="s">
         <v>132</v>
@@ -18023,14 +18028,14 @@
     </row>
     <row r="36" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A36" s="38" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="B36" s="38" t="s">
         <v>132</v>
       </c>
       <c r="C36" s="36">
         <f>MIN('Budget 36 mois'!E80:AN80)</f>
-        <v>-52928.892857142862</v>
+        <v>10071.107142857145</v>
       </c>
       <c r="D36" s="64"/>
       <c r="E36" s="64"/>
@@ -18042,7 +18047,7 @@
     </row>
     <row r="37" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="B37"/>
       <c r="C37" s="70">
@@ -18059,22 +18064,22 @@
     </row>
     <row r="38" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="B38" t="s">
         <v>132</v>
       </c>
       <c r="C38" s="64">
         <f>'Budget 36 mois'!P80</f>
-        <v>-8551.1785714285943</v>
+        <v>54448.821428571413</v>
       </c>
       <c r="D38" s="64">
         <f>'Budget 36 mois'!AB80</f>
-        <v>433353.49647619051</v>
+        <v>496353.49647619051</v>
       </c>
       <c r="E38" s="64">
         <f>'Budget 36 mois'!AN80</f>
-        <v>808460.35847619059</v>
+        <v>871460.35847619059</v>
       </c>
       <c r="F38"/>
       <c r="G38"/>
@@ -18084,7 +18089,7 @@
     </row>
     <row r="39" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="B39" t="s">
         <v>132</v>
@@ -18121,7 +18126,7 @@
     </row>
     <row r="41" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A41" s="60" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="B41"/>
       <c r="C41"/>
@@ -18380,12 +18385,12 @@
   <sheetData>
     <row r="1" spans="1:9" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="59" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="60" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
@@ -18401,24 +18406,24 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="C5" s="74">
         <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="C6" s="74">
         <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="42" customHeight="1" x14ac:dyDescent="0.35">
@@ -18426,16 +18431,16 @@
         <v>26</v>
       </c>
       <c r="B7" s="62" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="C7" s="62" t="s">
         <v>139</v>
       </c>
       <c r="D7" s="62" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="E7" s="62" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="F7" s="62" t="s">
         <v>140</v>
@@ -18512,7 +18517,7 @@
         <v>82</v>
       </c>
       <c r="I9" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
@@ -18545,12 +18550,12 @@
         <v>82</v>
       </c>
       <c r="I10" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="34" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="B11" s="34">
         <v>1</v>
@@ -18577,7 +18582,7 @@
         <v>82</v>
       </c>
       <c r="I11" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
@@ -18605,7 +18610,7 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="60" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
     </row>
   </sheetData>

</xml_diff>